<commit_message>
Add Uda coop approach briefing, phone script label, Aizu school DC reference, Uda audit PDF; update Oba village data
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/reference/mitsue_village_forestry_data_oba_2026-10-27.xlsx
+++ b/docs/reference/mitsue_village_forestry_data_oba_2026-10-27.xlsx
@@ -9,14 +9,15 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bids_FY2026" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ForestTax_Programs" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ForestTax_Totals" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Machinery_Loan" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Oba_Answers" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bids_Construction_FY2026" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ForestTax_Programs" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ForestTax_Totals" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Machinery_Loan" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Oba_Answers" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Bids_FY2026'!$A$1:$I$37</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'ForestTax_Programs'!$A$1:$E$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'ForestTax_Programs'!$A$1:$E$27</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -76,7 +77,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -113,6 +114,7 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -478,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -590,6 +592,18 @@
       <c r="B9" s="2" t="inlineStr">
         <is>
           <t>Figures were read from PDF text extraction; the older tax tables (FY2019-FY2022) are large survey forms with cut-off columns. Verify against the PDFs before quoting. FY2021 PDF (20230214.pdf) is an image with no text and was not read.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Update 2026-10-28</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Re-checked village site: no new service-bid results after 10/15. Added sheet Bids_Construction_FY2026 (7 construction tenders, Apr–Oct 2026, none forestry). 10/20 results page and 10月工事発注見通し (road/bridge works only) reviewed.</t>
         </is>
       </c>
     </row>
@@ -2114,6 +2128,1532 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:I40"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Bid date</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Project (業務名)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Reserve price ¥ (予定価格, tax-excl. unless noted)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Bidder</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Bid ¥</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Bid / reserve</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Source PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>みつえ青少年旅行村             ウッドデッキ改築工事</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>御杖村大字神末1790番地 みつえ青少年旅行村</t>
+        </is>
+      </c>
+      <c r="D2" s="14" t="n">
+        <v>4149200</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>株式会社 立花商会 代表取締役 立花 正富</t>
+        </is>
+      </c>
+      <c r="F2" s="14" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="G2" s="13">
+        <f>IF(F2="","",F2/D2)</f>
+        <v/>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>落札</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>kekka_20260410.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>(same)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>(same)</t>
+        </is>
+      </c>
+      <c r="D3" s="14" t="n">
+        <v>4149200</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>中村建築 中村 公</t>
+        </is>
+      </c>
+      <c r="F3" s="14" t="n">
+        <v>4140000</v>
+      </c>
+      <c r="G3" s="13">
+        <f>IF(F3="","",F3/D3)</f>
+        <v/>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>kekka_20260410.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>(same)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>(same)</t>
+        </is>
+      </c>
+      <c r="D4" s="14" t="n">
+        <v>4149200</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>株式会社 坂口組 代表取締役 坂口 明男</t>
+        </is>
+      </c>
+      <c r="F4" s="14" t="n">
+        <v>4200000</v>
+      </c>
+      <c r="G4" s="13">
+        <f>IF(F4="","",F4/D4)</f>
+        <v/>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>kekka_20260410.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>(same)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>(same)</t>
+        </is>
+      </c>
+      <c r="D5" s="14" t="n">
+        <v>4149200</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>株式会社 坂本総建 代表取締役 坂本 大輔</t>
+        </is>
+      </c>
+      <c r="F5" s="14" t="n">
+        <v>4200000</v>
+      </c>
+      <c r="G5" s="13">
+        <f>IF(F5="","",F5/D5)</f>
+        <v/>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>kekka_20260410.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>みつえ青少年旅行村新規サイト敷地整備工事</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>御杖村大字神末 地内</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="n">
+        <v>70327000</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>（株）坂口組 代表取締役 坂口明男</t>
+        </is>
+      </c>
+      <c r="F6" s="14" t="n">
+        <v>67000000</v>
+      </c>
+      <c r="G6" s="13">
+        <f>IF(F6="","",F6/D6)</f>
+        <v/>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>落札</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>kekka_20260522.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>(same)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>(same)</t>
+        </is>
+      </c>
+      <c r="D7" s="14" t="n">
+        <v>70327000</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>中嶋建設（株） 代表取締役 中嶋敏治</t>
+        </is>
+      </c>
+      <c r="F7" s="14" t="n">
+        <v>68650000</v>
+      </c>
+      <c r="G7" s="13">
+        <f>IF(F7="","",F7/D7)</f>
+        <v/>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>kekka_20260522.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>(same)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>(same)</t>
+        </is>
+      </c>
+      <c r="D8" s="14" t="n">
+        <v>70327000</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>（株）山田土木 代表取締役 山田浩之</t>
+        </is>
+      </c>
+      <c r="F8" s="14" t="n">
+        <v>69000000</v>
+      </c>
+      <c r="G8" s="13">
+        <f>IF(F8="","",F8/D8)</f>
+        <v/>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>kekka_20260522.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>御杖村保健センターＬＥＤ照明改修工事</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>御杖村大字菅野１５８１ 御杖村保健センター</t>
+        </is>
+      </c>
+      <c r="D9" s="14" t="n">
+        <v>34211000</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>松田電気工業(株)</t>
+        </is>
+      </c>
+      <c r="F9" s="14" t="n">
+        <v>29500000</v>
+      </c>
+      <c r="G9" s="13">
+        <f>IF(F9="","",F9/D9)</f>
+        <v/>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>落札</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>kekka_20260723.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>(same)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>(same)</t>
+        </is>
+      </c>
+      <c r="D10" s="14" t="n">
+        <v>34211000</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>(株)きんでん奈良支店</t>
+        </is>
+      </c>
+      <c r="F10" s="14" t="n">
+        <v>29800000</v>
+      </c>
+      <c r="G10" s="13">
+        <f>IF(F10="","",F10/D10)</f>
+        <v/>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>kekka_20260723.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>(same)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>(same)</t>
+        </is>
+      </c>
+      <c r="D11" s="14" t="n">
+        <v>34211000</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>吉田機電(株)</t>
+        </is>
+      </c>
+      <c r="F11" s="14" t="n">
+        <v>32500000</v>
+      </c>
+      <c r="G11" s="13">
+        <f>IF(F11="","",F11/D11)</f>
+        <v/>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>kekka_20260723.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>(same)</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>(same)</t>
+        </is>
+      </c>
+      <c r="D12" s="14" t="n">
+        <v>34211000</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>奈良文庫電気設備(株)</t>
+        </is>
+      </c>
+      <c r="F12" s="14" t="n">
+        <v>32800000</v>
+      </c>
+      <c r="G12" s="13">
+        <f>IF(F12="","",F12/D12)</f>
+        <v/>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>kekka_20260723.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>(same)</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>(same)</t>
+        </is>
+      </c>
+      <c r="D13" s="14" t="n">
+        <v>34211000</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>信貴商事(株)</t>
+        </is>
+      </c>
+      <c r="F13" s="14" t="n">
+        <v>35000000</v>
+      </c>
+      <c r="G13" s="13">
+        <f>IF(F13="","",F13/D13)</f>
+        <v/>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>kekka_20260723.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>御杖村山村開発センターＬＥＤ照明改修工事</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>御杖村大字菅野３６８ 御杖村山村開発センター</t>
+        </is>
+      </c>
+      <c r="D14" s="14" t="n">
+        <v>27006000</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>(株)きんでん奈良支店</t>
+        </is>
+      </c>
+      <c r="F14" s="14" t="n">
+        <v>24800000</v>
+      </c>
+      <c r="G14" s="13">
+        <f>IF(F14="","",F14/D14)</f>
+        <v/>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>落札</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>kekka_20260723.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>(same)</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>(same)</t>
+        </is>
+      </c>
+      <c r="D15" s="14" t="n">
+        <v>27006000</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>松田電気工業(株)</t>
+        </is>
+      </c>
+      <c r="F15" s="14" t="n">
+        <v>25000000</v>
+      </c>
+      <c r="G15" s="13">
+        <f>IF(F15="","",F15/D15)</f>
+        <v/>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>kekka_20260723.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>(same)</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>(same)</t>
+        </is>
+      </c>
+      <c r="D16" s="14" t="n">
+        <v>27006000</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>吉田機電(株)</t>
+        </is>
+      </c>
+      <c r="F16" s="14" t="n">
+        <v>25500000</v>
+      </c>
+      <c r="G16" s="13">
+        <f>IF(F16="","",F16/D16)</f>
+        <v/>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>kekka_20260723.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>(same)</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>(same)</t>
+        </is>
+      </c>
+      <c r="D17" s="14" t="n">
+        <v>27006000</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>奈良文庫電気設備(株)</t>
+        </is>
+      </c>
+      <c r="F17" s="14" t="n">
+        <v>25800000</v>
+      </c>
+      <c r="G17" s="13">
+        <f>IF(F17="","",F17/D17)</f>
+        <v/>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>kekka_20260723.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>(same)</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>(same)</t>
+        </is>
+      </c>
+      <c r="D18" s="14" t="n">
+        <v>27006000</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>信貴商事(株)</t>
+        </is>
+      </c>
+      <c r="F18" s="14" t="n">
+        <v>27000000</v>
+      </c>
+      <c r="G18" s="13">
+        <f>IF(F18="","",F18/D18)</f>
+        <v/>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>kekka_20260723.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>御杖保育所中庭ウッドデッキ改修工事</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>御杖村大字大字土屋原1479番地の1</t>
+        </is>
+      </c>
+      <c r="D19" s="14" t="n">
+        <v>4893000</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>中村建築 中村 公</t>
+        </is>
+      </c>
+      <c r="F19" s="14" t="n">
+        <v>4880000</v>
+      </c>
+      <c r="G19" s="13">
+        <f>IF(F19="","",F19/D19)</f>
+        <v/>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>落札</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>kekka_20260810.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>(same)</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>(same)</t>
+        </is>
+      </c>
+      <c r="D20" s="14" t="n">
+        <v>4893000</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>株式会社立花商会 代表取締役 立花 正富</t>
+        </is>
+      </c>
+      <c r="F20" s="14" t="n">
+        <v>4900000</v>
+      </c>
+      <c r="G20" s="13">
+        <f>IF(F20="","",F20/D20)</f>
+        <v/>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>kekka_20260810.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>(same)</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>(same)</t>
+        </is>
+      </c>
+      <c r="D21" s="14" t="n">
+        <v>4893000</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>株式会社坂口組 代表取締役 坂口 明男</t>
+        </is>
+      </c>
+      <c r="F21" s="14" t="n">
+        <v>5050000</v>
+      </c>
+      <c r="G21" s="13">
+        <f>IF(F21="","",F21/D21)</f>
+        <v/>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>kekka_20260810.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>(same)</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>(same)</t>
+        </is>
+      </c>
+      <c r="D22" s="14" t="n">
+        <v>4893000</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>株式会社坂本総建 代表取締役 坂本 大輔</t>
+        </is>
+      </c>
+      <c r="F22" s="14" t="n">
+        <v>5100000</v>
+      </c>
+      <c r="G22" s="13">
+        <f>IF(F22="","",F22/D22)</f>
+        <v/>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>kekka_20260810.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>令和８年度 菅野地区配水管布設替工事</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>御杖村大字 菅野 地内</t>
+        </is>
+      </c>
+      <c r="D23" s="14" t="n">
+        <v>44630000</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>中嶋建設(株) 中嶋敏治</t>
+        </is>
+      </c>
+      <c r="F23" s="14" t="n">
+        <v>44000000</v>
+      </c>
+      <c r="G23" s="13">
+        <f>IF(F23="","",F23/D23)</f>
+        <v/>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>落札</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>kekka_20260814.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>(same)</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>(same)</t>
+        </is>
+      </c>
+      <c r="D24" s="14" t="n">
+        <v>44630000</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>(株)坂口組 坂口明男</t>
+        </is>
+      </c>
+      <c r="F24" s="14" t="n">
+        <v>44200000</v>
+      </c>
+      <c r="G24" s="13">
+        <f>IF(F24="","",F24/D24)</f>
+        <v/>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>kekka_20260814.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>(same)</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>(same)</t>
+        </is>
+      </c>
+      <c r="D25" s="14" t="n">
+        <v>44630000</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>(株)山田土木 山田浩之</t>
+        </is>
+      </c>
+      <c r="F25" s="14" t="n">
+        <v>44500000</v>
+      </c>
+      <c r="G25" s="13">
+        <f>IF(F25="","",F25/D25)</f>
+        <v/>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>kekka_20260814.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>防災･安全交付金事業 村道中村線舗装補修工事</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>御杖村大字 土屋原 地内</t>
+        </is>
+      </c>
+      <c r="D26" s="14" t="n"/>
+      <c r="F26" s="14" t="n"/>
+      <c r="G26" s="13" t="n"/>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>入札取消し (予定価格の誤り; re-bid 2026-08-27)</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>kekka_20260814.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>防災･安全交付金事業 村道西川川合敷津線(神末工区)舗装補修工事</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>御杖村大字 神末 地内</t>
+        </is>
+      </c>
+      <c r="D27" s="14" t="n">
+        <v>7077000</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>共 今西組 今西 ちえ子</t>
+        </is>
+      </c>
+      <c r="F27" s="14" t="n">
+        <v>6790000</v>
+      </c>
+      <c r="G27" s="13">
+        <f>IF(F27="","",F27/D27)</f>
+        <v/>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>落札</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>kekka_20260814.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>(same)</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>(same)</t>
+        </is>
+      </c>
+      <c r="D28" s="14" t="n">
+        <v>7077000</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>株式会社木村組 木村 ますみ</t>
+        </is>
+      </c>
+      <c r="F28" s="14" t="n">
+        <v>6900000</v>
+      </c>
+      <c r="G28" s="13">
+        <f>IF(F28="","",F28/D28)</f>
+        <v/>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>kekka_20260814.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>(same)</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>(same)</t>
+        </is>
+      </c>
+      <c r="D29" s="14" t="n">
+        <v>7077000</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>株式会社山田土木 山田 浩之</t>
+        </is>
+      </c>
+      <c r="F29" s="14" t="n">
+        <v>7000000</v>
+      </c>
+      <c r="G29" s="13">
+        <f>IF(F29="","",F29/D29)</f>
+        <v/>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>kekka_20260814.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>(same)</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>(same)</t>
+        </is>
+      </c>
+      <c r="D30" s="14" t="n">
+        <v>7077000</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>株式会社坂口組 坂口 明男</t>
+        </is>
+      </c>
+      <c r="F30" s="14" t="n">
+        <v>7000000</v>
+      </c>
+      <c r="G30" s="13">
+        <f>IF(F30="","",F30/D30)</f>
+        <v/>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>kekka_20260814.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>(same)</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>(same)</t>
+        </is>
+      </c>
+      <c r="D31" s="14" t="n">
+        <v>7077000</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>中嶋建設株式会社 中嶋 敏治</t>
+        </is>
+      </c>
+      <c r="F31" s="14" t="n">
+        <v>7035000</v>
+      </c>
+      <c r="G31" s="13">
+        <f>IF(F31="","",F31/D31)</f>
+        <v/>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>kekka_20260814.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>防災･安全交付金事業 村道中村線舗装補修工事</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>御杖村大字 土屋原 地内</t>
+        </is>
+      </c>
+      <c r="D32" s="14" t="n">
+        <v>20452000</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>株式会社山田土木 山田 浩之</t>
+        </is>
+      </c>
+      <c r="F32" s="14" t="n">
+        <v>20000000</v>
+      </c>
+      <c r="G32" s="13">
+        <f>IF(F32="","",F32/D32)</f>
+        <v/>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>落札</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>kekka_20260827.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>(same)</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>(same)</t>
+        </is>
+      </c>
+      <c r="D33" s="14" t="n">
+        <v>20452000</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>中嶋建設株式会社 中嶋 敏治</t>
+        </is>
+      </c>
+      <c r="F33" s="14" t="n">
+        <v>20250000</v>
+      </c>
+      <c r="G33" s="13">
+        <f>IF(F33="","",F33/D33)</f>
+        <v/>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>kekka_20260827.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>(same)</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>(same)</t>
+        </is>
+      </c>
+      <c r="D34" s="14" t="n">
+        <v>20452000</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>株式会社坂口組 坂口 明男</t>
+        </is>
+      </c>
+      <c r="F34" s="14" t="n">
+        <v>20300000</v>
+      </c>
+      <c r="G34" s="13">
+        <f>IF(F34="","",F34/D34)</f>
+        <v/>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>kekka_20260827.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>村道脇谷中野線 部分改良工事</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>御杖村大字 神末 地内</t>
+        </is>
+      </c>
+      <c r="D35" s="14" t="n">
+        <v>8415000</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>株式会社木村組 木村 ますみ</t>
+        </is>
+      </c>
+      <c r="F35" s="14" t="n">
+        <v>8000000</v>
+      </c>
+      <c r="G35" s="13">
+        <f>IF(F35="","",F35/D35)</f>
+        <v/>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>落札</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>kekka_20261015.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>(same)</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>(same)</t>
+        </is>
+      </c>
+      <c r="D36" s="14" t="n">
+        <v>8415000</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>株式会社坂口組 坂口 明男</t>
+        </is>
+      </c>
+      <c r="F36" s="14" t="n">
+        <v>8200000</v>
+      </c>
+      <c r="G36" s="13">
+        <f>IF(F36="","",F36/D36)</f>
+        <v/>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>kekka_20261015.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>(same)</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>(same)</t>
+        </is>
+      </c>
+      <c r="D37" s="14" t="n">
+        <v>8415000</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>共 今西組 今西 ちえ子</t>
+        </is>
+      </c>
+      <c r="F37" s="14" t="n">
+        <v>8200000</v>
+      </c>
+      <c r="G37" s="13">
+        <f>IF(F37="","",F37/D37)</f>
+        <v/>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>kekka_20261015.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>(same)</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>(same)</t>
+        </is>
+      </c>
+      <c r="D38" s="14" t="n">
+        <v>8415000</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>中嶋建設株式会社 中嶋 敏治</t>
+        </is>
+      </c>
+      <c r="F38" s="14" t="n">
+        <v>8250000</v>
+      </c>
+      <c r="G38" s="13">
+        <f>IF(F38="","",F38/D38)</f>
+        <v/>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>kekka_20261015.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>(same)</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>(same)</t>
+        </is>
+      </c>
+      <c r="D39" s="14" t="n">
+        <v>8415000</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>株式会社山田土木 山田 浩之</t>
+        </is>
+      </c>
+      <c r="F39" s="14" t="n">
+        <v>8300000</v>
+      </c>
+      <c r="G39" s="13">
+        <f>IF(F39="","",F39/D39)</f>
+        <v/>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>kekka_20261015.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Note: all 指名競争入札. Source: construction (建設工事) results, https://www.vill.mitsue.nara.jp/material/files/group/10/ (kekka_*.pdf). 契約額 = bid +10% tax. 2026-08-14 中村線 bid cancelled (reserve price error in published form), re-bid 8/27. Added 2026-10-28; no forestry work among these.</t>
+        </is>
+      </c>
+      <c r="D40" s="14" t="n"/>
+      <c r="F40" s="14" t="n"/>
+      <c r="G40" s="13" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2757,7 +4297,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2915,7 +4455,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3104,7 +4644,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>